<commit_message>
repo clean up 2
</commit_message>
<xml_diff>
--- a/source_data/GLM_Figures.xlsx
+++ b/source_data/GLM_Figures.xlsx
@@ -48,7 +48,7 @@
     <t>Pooled state+month FE IRRs for temperature and rainfall, by model family (* = Significant)</t>
   </si>
   <si>
-    <t>outputs/glm_*_pooled_fe.csv; plot_glm_results.R</t>
+    <t>outputs/regression/glm_*_pooled_fe.csv; plot_glm_results.R</t>
   </si>
   <si>
     <t>glm_fig2_state_heatmap</t>
@@ -57,7 +57,7 @@
     <t>Per-state NegBin IRRs (heatmap colour = log2 IRR)</t>
   </si>
   <si>
-    <t>outputs/glm_negbin_per_state.csv; plot_glm_results.R</t>
+    <t>outputs/regression/glm_negbin_per_state.csv; plot_glm_results.R</t>
   </si>
   <si>
     <t>glm_fig3_lag_profile</t>
@@ -66,7 +66,7 @@
     <t>Median and IQR of per-state NegBin IRRs by lag</t>
   </si>
   <si>
-    <t>outputs/glm_negbin_lagged.csv; plot_glm_results.R</t>
+    <t>outputs/regression/glm_negbin_lagged.csv; plot_glm_results.R</t>
   </si>
   <si>
     <t>glm_fig4_aic</t>
@@ -75,7 +75,7 @@
     <t>Median AIC across states per family × specification × virus</t>
   </si>
   <si>
-    <t>outputs/glm_*_*.csv; plot_glm_results.R</t>
+    <t>outputs/regression/glm_*_*.csv; plot_glm_results.R</t>
   </si>
   <si>
     <t>glm_fig5_forest</t>

</xml_diff>